<commit_message>
Add temporary Excel file for Jabulane Poulo April final week
</commit_message>
<xml_diff>
--- a/Projects/Timesheet/Jabulane_Poulo/Jabulane_Poulo_April_FinalWeek.xlsx
+++ b/Projects/Timesheet/Jabulane_Poulo/Jabulane_Poulo_April_FinalWeek.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_JabulanePoulo_2026\Projects\Timesheet\Jabulane_Poulo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B76767F-34EA-4DCF-9E5B-F271BA29BF7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{011C515B-409D-4984-9758-4B7B87186AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1C8F8026-B005-4B08-94D3-371A77F74D8F}"/>
   </bookViews>
@@ -1929,28 +1929,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1966,6 +1951,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3629,7 +3629,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>57</v>
+        <v>125</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27" t="s">
@@ -12162,27 +12162,27 @@
       <c r="F7" s="85"/>
     </row>
     <row r="8" spans="1:15" ht="27.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="132" t="s">
+      <c r="A8" s="135" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="132"/>
-      <c r="C8" s="132"/>
-      <c r="D8" s="132"/>
-      <c r="E8" s="132"/>
-      <c r="F8" s="132"/>
+      <c r="B8" s="135"/>
+      <c r="C8" s="135"/>
+      <c r="D8" s="135"/>
+      <c r="E8" s="135"/>
+      <c r="F8" s="135"/>
     </row>
     <row r="9" spans="1:15" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="82" t="s">
         <v>170</v>
       </c>
-      <c r="B9" s="129" t="s">
+      <c r="B9" s="138" t="s">
         <v>167</v>
       </c>
-      <c r="C9" s="130"/>
-      <c r="D9" s="129" t="s">
+      <c r="C9" s="139"/>
+      <c r="D9" s="138" t="s">
         <v>94</v>
       </c>
-      <c r="E9" s="130"/>
+      <c r="E9" s="139"/>
       <c r="F9" s="83" t="s">
         <v>95</v>
       </c>
@@ -12191,103 +12191,103 @@
       <c r="A10" s="78">
         <v>46113</v>
       </c>
-      <c r="B10" s="131" t="s">
+      <c r="B10" s="129" t="s">
         <v>168</v>
       </c>
-      <c r="C10" s="131"/>
-      <c r="D10" s="131" t="s">
+      <c r="C10" s="129"/>
+      <c r="D10" s="129" t="s">
         <v>123</v>
       </c>
-      <c r="E10" s="131"/>
+      <c r="E10" s="129"/>
       <c r="F10" s="77">
         <v>200</v>
       </c>
-      <c r="G10" s="127" t="s">
+      <c r="G10" s="136" t="s">
         <v>169</v>
       </c>
-      <c r="H10" s="128"/>
-      <c r="I10" s="128"/>
-      <c r="J10" s="128"/>
-      <c r="K10" s="128"/>
-      <c r="L10" s="128"/>
-      <c r="M10" s="128"/>
-      <c r="N10" s="128"/>
-      <c r="O10" s="128"/>
+      <c r="H10" s="137"/>
+      <c r="I10" s="137"/>
+      <c r="J10" s="137"/>
+      <c r="K10" s="137"/>
+      <c r="L10" s="137"/>
+      <c r="M10" s="137"/>
+      <c r="N10" s="137"/>
+      <c r="O10" s="137"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="78">
         <v>46113</v>
       </c>
-      <c r="B11" s="133" t="s">
+      <c r="B11" s="127" t="s">
         <v>171</v>
       </c>
-      <c r="C11" s="134"/>
-      <c r="D11" s="131" t="s">
+      <c r="C11" s="128"/>
+      <c r="D11" s="129" t="s">
         <v>128</v>
       </c>
-      <c r="E11" s="131"/>
+      <c r="E11" s="129"/>
       <c r="F11" s="77"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="78">
         <v>46113</v>
       </c>
-      <c r="B12" s="133" t="s">
+      <c r="B12" s="127" t="s">
         <v>172</v>
       </c>
-      <c r="C12" s="134"/>
-      <c r="D12" s="131"/>
-      <c r="E12" s="131"/>
+      <c r="C12" s="128"/>
+      <c r="D12" s="129"/>
+      <c r="E12" s="129"/>
       <c r="F12" s="77"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="78">
         <v>46113</v>
       </c>
-      <c r="B13" s="133"/>
-      <c r="C13" s="134"/>
-      <c r="D13" s="131"/>
-      <c r="E13" s="131"/>
+      <c r="B13" s="127"/>
+      <c r="C13" s="128"/>
+      <c r="D13" s="129"/>
+      <c r="E13" s="129"/>
       <c r="F13" s="77"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="78">
         <v>46113</v>
       </c>
-      <c r="B14" s="133"/>
-      <c r="C14" s="134"/>
-      <c r="D14" s="131"/>
-      <c r="E14" s="131"/>
+      <c r="B14" s="127"/>
+      <c r="C14" s="128"/>
+      <c r="D14" s="129"/>
+      <c r="E14" s="129"/>
       <c r="F14" s="77"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="78">
         <v>46113</v>
       </c>
-      <c r="B15" s="138"/>
-      <c r="C15" s="139"/>
-      <c r="D15" s="131"/>
-      <c r="E15" s="131"/>
+      <c r="B15" s="133"/>
+      <c r="C15" s="134"/>
+      <c r="D15" s="129"/>
+      <c r="E15" s="129"/>
       <c r="F15" s="77"/>
     </row>
     <row r="16" spans="1:15" ht="13.2" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="78">
         <v>46113</v>
       </c>
-      <c r="B16" s="133"/>
-      <c r="C16" s="134"/>
-      <c r="D16" s="131"/>
-      <c r="E16" s="131"/>
+      <c r="B16" s="127"/>
+      <c r="C16" s="128"/>
+      <c r="D16" s="129"/>
+      <c r="E16" s="129"/>
       <c r="F16" s="77"/>
     </row>
     <row r="17" spans="1:6" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="135" t="s">
+      <c r="A17" s="130" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="136"/>
-      <c r="C17" s="136"/>
-      <c r="D17" s="136"/>
-      <c r="E17" s="137"/>
+      <c r="B17" s="131"/>
+      <c r="C17" s="131"/>
+      <c r="D17" s="131"/>
+      <c r="E17" s="132"/>
       <c r="F17" s="76">
         <f>SUM(F10:F16)</f>
         <v>200</v>
@@ -12303,6 +12303,16 @@
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="G10:O10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:E12"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="A17:E17"/>
@@ -12312,16 +12322,6 @@
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D16:E16"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G10:O10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7 D18" xr:uid="{517DF1E8-3052-48CF-9AE1-C19E6ECB6686}">
@@ -13336,21 +13336,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD10A028B4ACBB47B37340D8D4079B36" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="436e80374471046821afb96e56969fce">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="606bf0c3-7c02-4ad1-9a2b-bad21eeec9a2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="819cb4b524acab89028d2f2d821df341" ns2:_="">
     <xsd:import namespace="606bf0c3-7c02-4ad1-9a2b-bad21eeec9a2"/>
@@ -13488,24 +13473,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D445429-43EF-4578-A593-6E166DDD94D2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBA7CA51-3876-42E5-9D60-4320955E597F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84037CEB-E5D3-4F40-B93D-B68754BA7EB6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13523,6 +13506,23 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBA7CA51-3876-42E5-9D60-4320955E597F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D445429-43EF-4578-A593-6E166DDD94D2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{5138fff4-6130-46cf-adb5-ec5d984d54d5}" enabled="1" method="Privileged" siteId="{174c7352-9c5c-4558-b848-be140b444e7d}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Update Jabulane Poulo April final week Excel file
</commit_message>
<xml_diff>
--- a/Projects/Timesheet/Jabulane_Poulo/Jabulane_Poulo_April_FinalWeek.xlsx
+++ b/Projects/Timesheet/Jabulane_Poulo/Jabulane_Poulo_April_FinalWeek.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_JabulanePoulo_2026\Projects\Timesheet\Jabulane_Poulo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{011C515B-409D-4984-9758-4B7B87186AE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48E13CB4-2E81-4D6F-B0C0-4ABDCFB946FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1C8F8026-B005-4B08-94D3-371A77F74D8F}"/>
   </bookViews>
@@ -1929,13 +1929,28 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1951,21 +1966,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3629,7 +3629,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27" t="s">
@@ -12162,27 +12162,27 @@
       <c r="F7" s="85"/>
     </row>
     <row r="8" spans="1:15" ht="27.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="135" t="s">
+      <c r="A8" s="132" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="135"/>
-      <c r="C8" s="135"/>
-      <c r="D8" s="135"/>
-      <c r="E8" s="135"/>
-      <c r="F8" s="135"/>
+      <c r="B8" s="132"/>
+      <c r="C8" s="132"/>
+      <c r="D8" s="132"/>
+      <c r="E8" s="132"/>
+      <c r="F8" s="132"/>
     </row>
     <row r="9" spans="1:15" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="82" t="s">
         <v>170</v>
       </c>
-      <c r="B9" s="138" t="s">
+      <c r="B9" s="129" t="s">
         <v>167</v>
       </c>
-      <c r="C9" s="139"/>
-      <c r="D9" s="138" t="s">
+      <c r="C9" s="130"/>
+      <c r="D9" s="129" t="s">
         <v>94</v>
       </c>
-      <c r="E9" s="139"/>
+      <c r="E9" s="130"/>
       <c r="F9" s="83" t="s">
         <v>95</v>
       </c>
@@ -12191,103 +12191,103 @@
       <c r="A10" s="78">
         <v>46113</v>
       </c>
-      <c r="B10" s="129" t="s">
+      <c r="B10" s="131" t="s">
         <v>168</v>
       </c>
-      <c r="C10" s="129"/>
-      <c r="D10" s="129" t="s">
+      <c r="C10" s="131"/>
+      <c r="D10" s="131" t="s">
         <v>123</v>
       </c>
-      <c r="E10" s="129"/>
+      <c r="E10" s="131"/>
       <c r="F10" s="77">
         <v>200</v>
       </c>
-      <c r="G10" s="136" t="s">
+      <c r="G10" s="127" t="s">
         <v>169</v>
       </c>
-      <c r="H10" s="137"/>
-      <c r="I10" s="137"/>
-      <c r="J10" s="137"/>
-      <c r="K10" s="137"/>
-      <c r="L10" s="137"/>
-      <c r="M10" s="137"/>
-      <c r="N10" s="137"/>
-      <c r="O10" s="137"/>
+      <c r="H10" s="128"/>
+      <c r="I10" s="128"/>
+      <c r="J10" s="128"/>
+      <c r="K10" s="128"/>
+      <c r="L10" s="128"/>
+      <c r="M10" s="128"/>
+      <c r="N10" s="128"/>
+      <c r="O10" s="128"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="78">
         <v>46113</v>
       </c>
-      <c r="B11" s="127" t="s">
+      <c r="B11" s="133" t="s">
         <v>171</v>
       </c>
-      <c r="C11" s="128"/>
-      <c r="D11" s="129" t="s">
+      <c r="C11" s="134"/>
+      <c r="D11" s="131" t="s">
         <v>128</v>
       </c>
-      <c r="E11" s="129"/>
+      <c r="E11" s="131"/>
       <c r="F11" s="77"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="78">
         <v>46113</v>
       </c>
-      <c r="B12" s="127" t="s">
+      <c r="B12" s="133" t="s">
         <v>172</v>
       </c>
-      <c r="C12" s="128"/>
-      <c r="D12" s="129"/>
-      <c r="E12" s="129"/>
+      <c r="C12" s="134"/>
+      <c r="D12" s="131"/>
+      <c r="E12" s="131"/>
       <c r="F12" s="77"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="78">
         <v>46113</v>
       </c>
-      <c r="B13" s="127"/>
-      <c r="C13" s="128"/>
-      <c r="D13" s="129"/>
-      <c r="E13" s="129"/>
+      <c r="B13" s="133"/>
+      <c r="C13" s="134"/>
+      <c r="D13" s="131"/>
+      <c r="E13" s="131"/>
       <c r="F13" s="77"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="78">
         <v>46113</v>
       </c>
-      <c r="B14" s="127"/>
-      <c r="C14" s="128"/>
-      <c r="D14" s="129"/>
-      <c r="E14" s="129"/>
+      <c r="B14" s="133"/>
+      <c r="C14" s="134"/>
+      <c r="D14" s="131"/>
+      <c r="E14" s="131"/>
       <c r="F14" s="77"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="78">
         <v>46113</v>
       </c>
-      <c r="B15" s="133"/>
-      <c r="C15" s="134"/>
-      <c r="D15" s="129"/>
-      <c r="E15" s="129"/>
+      <c r="B15" s="138"/>
+      <c r="C15" s="139"/>
+      <c r="D15" s="131"/>
+      <c r="E15" s="131"/>
       <c r="F15" s="77"/>
     </row>
     <row r="16" spans="1:15" ht="13.2" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="78">
         <v>46113</v>
       </c>
-      <c r="B16" s="127"/>
-      <c r="C16" s="128"/>
-      <c r="D16" s="129"/>
-      <c r="E16" s="129"/>
+      <c r="B16" s="133"/>
+      <c r="C16" s="134"/>
+      <c r="D16" s="131"/>
+      <c r="E16" s="131"/>
       <c r="F16" s="77"/>
     </row>
     <row r="17" spans="1:6" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="130" t="s">
+      <c r="A17" s="135" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="131"/>
-      <c r="C17" s="131"/>
-      <c r="D17" s="131"/>
-      <c r="E17" s="132"/>
+      <c r="B17" s="136"/>
+      <c r="C17" s="136"/>
+      <c r="D17" s="136"/>
+      <c r="E17" s="137"/>
       <c r="F17" s="76">
         <f>SUM(F10:F16)</f>
         <v>200</v>
@@ -12303,16 +12303,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="G10:O10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:E12"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="A17:E17"/>
@@ -12322,6 +12312,16 @@
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G10:O10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7 D18" xr:uid="{517DF1E8-3052-48CF-9AE1-C19E6ECB6686}">
@@ -13336,6 +13336,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD10A028B4ACBB47B37340D8D4079B36" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="436e80374471046821afb96e56969fce">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="606bf0c3-7c02-4ad1-9a2b-bad21eeec9a2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="819cb4b524acab89028d2f2d821df341" ns2:_="">
     <xsd:import namespace="606bf0c3-7c02-4ad1-9a2b-bad21eeec9a2"/>
@@ -13473,22 +13488,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D445429-43EF-4578-A593-6E166DDD94D2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBA7CA51-3876-42E5-9D60-4320955E597F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84037CEB-E5D3-4F40-B93D-B68754BA7EB6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13506,23 +13523,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBA7CA51-3876-42E5-9D60-4320955E597F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D445429-43EF-4578-A593-6E166DDD94D2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{5138fff4-6130-46cf-adb5-ec5d984d54d5}" enabled="1" method="Privileged" siteId="{174c7352-9c5c-4558-b848-be140b444e7d}" contentBits="2" removed="0"/>

</xml_diff>

<commit_message>
Update Timesheet Migration project files and Excel data
</commit_message>
<xml_diff>
--- a/Projects/Timesheet/Jabulane_Poulo/Jabulane_Poulo_April_FinalWeek.xlsx
+++ b/Projects/Timesheet/Jabulane_Poulo/Jabulane_Poulo_April_FinalWeek.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_JabulanePoulo_2026\Projects\Timesheet\Jabulane_Poulo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{861FF522-721F-45D4-956B-0230E4B75EAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F526583-37F7-427C-925F-5B6A6BBDE374}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{1C8F8026-B005-4B08-94D3-371A77F74D8F}"/>
   </bookViews>
@@ -1929,13 +1929,28 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1951,21 +1966,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -3629,7 +3629,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>125</v>
+        <v>57</v>
       </c>
       <c r="D9" s="27"/>
       <c r="E9" s="27" t="s">
@@ -12162,27 +12162,27 @@
       <c r="F7" s="85"/>
     </row>
     <row r="8" spans="1:15" ht="27.45" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="135" t="s">
+      <c r="A8" s="132" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="135"/>
-      <c r="C8" s="135"/>
-      <c r="D8" s="135"/>
-      <c r="E8" s="135"/>
-      <c r="F8" s="135"/>
+      <c r="B8" s="132"/>
+      <c r="C8" s="132"/>
+      <c r="D8" s="132"/>
+      <c r="E8" s="132"/>
+      <c r="F8" s="132"/>
     </row>
     <row r="9" spans="1:15" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A9" s="82" t="s">
         <v>170</v>
       </c>
-      <c r="B9" s="138" t="s">
+      <c r="B9" s="129" t="s">
         <v>167</v>
       </c>
-      <c r="C9" s="139"/>
-      <c r="D9" s="138" t="s">
+      <c r="C9" s="130"/>
+      <c r="D9" s="129" t="s">
         <v>94</v>
       </c>
-      <c r="E9" s="139"/>
+      <c r="E9" s="130"/>
       <c r="F9" s="83" t="s">
         <v>95</v>
       </c>
@@ -12191,103 +12191,103 @@
       <c r="A10" s="78">
         <v>46113</v>
       </c>
-      <c r="B10" s="129" t="s">
+      <c r="B10" s="131" t="s">
         <v>168</v>
       </c>
-      <c r="C10" s="129"/>
-      <c r="D10" s="129" t="s">
+      <c r="C10" s="131"/>
+      <c r="D10" s="131" t="s">
         <v>123</v>
       </c>
-      <c r="E10" s="129"/>
+      <c r="E10" s="131"/>
       <c r="F10" s="77">
         <v>200</v>
       </c>
-      <c r="G10" s="136" t="s">
+      <c r="G10" s="127" t="s">
         <v>169</v>
       </c>
-      <c r="H10" s="137"/>
-      <c r="I10" s="137"/>
-      <c r="J10" s="137"/>
-      <c r="K10" s="137"/>
-      <c r="L10" s="137"/>
-      <c r="M10" s="137"/>
-      <c r="N10" s="137"/>
-      <c r="O10" s="137"/>
+      <c r="H10" s="128"/>
+      <c r="I10" s="128"/>
+      <c r="J10" s="128"/>
+      <c r="K10" s="128"/>
+      <c r="L10" s="128"/>
+      <c r="M10" s="128"/>
+      <c r="N10" s="128"/>
+      <c r="O10" s="128"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="78">
         <v>46113</v>
       </c>
-      <c r="B11" s="127" t="s">
+      <c r="B11" s="133" t="s">
         <v>171</v>
       </c>
-      <c r="C11" s="128"/>
-      <c r="D11" s="129" t="s">
+      <c r="C11" s="134"/>
+      <c r="D11" s="131" t="s">
         <v>128</v>
       </c>
-      <c r="E11" s="129"/>
+      <c r="E11" s="131"/>
       <c r="F11" s="77"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="78">
         <v>46113</v>
       </c>
-      <c r="B12" s="127" t="s">
+      <c r="B12" s="133" t="s">
         <v>172</v>
       </c>
-      <c r="C12" s="128"/>
-      <c r="D12" s="129"/>
-      <c r="E12" s="129"/>
+      <c r="C12" s="134"/>
+      <c r="D12" s="131"/>
+      <c r="E12" s="131"/>
       <c r="F12" s="77"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="78">
         <v>46113</v>
       </c>
-      <c r="B13" s="127"/>
-      <c r="C13" s="128"/>
-      <c r="D13" s="129"/>
-      <c r="E13" s="129"/>
+      <c r="B13" s="133"/>
+      <c r="C13" s="134"/>
+      <c r="D13" s="131"/>
+      <c r="E13" s="131"/>
       <c r="F13" s="77"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="78">
         <v>46113</v>
       </c>
-      <c r="B14" s="127"/>
-      <c r="C14" s="128"/>
-      <c r="D14" s="129"/>
-      <c r="E14" s="129"/>
+      <c r="B14" s="133"/>
+      <c r="C14" s="134"/>
+      <c r="D14" s="131"/>
+      <c r="E14" s="131"/>
       <c r="F14" s="77"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="78">
         <v>46113</v>
       </c>
-      <c r="B15" s="133"/>
-      <c r="C15" s="134"/>
-      <c r="D15" s="129"/>
-      <c r="E15" s="129"/>
+      <c r="B15" s="138"/>
+      <c r="C15" s="139"/>
+      <c r="D15" s="131"/>
+      <c r="E15" s="131"/>
       <c r="F15" s="77"/>
     </row>
     <row r="16" spans="1:15" ht="13.2" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="78">
         <v>46113</v>
       </c>
-      <c r="B16" s="127"/>
-      <c r="C16" s="128"/>
-      <c r="D16" s="129"/>
-      <c r="E16" s="129"/>
+      <c r="B16" s="133"/>
+      <c r="C16" s="134"/>
+      <c r="D16" s="131"/>
+      <c r="E16" s="131"/>
       <c r="F16" s="77"/>
     </row>
     <row r="17" spans="1:6" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="130" t="s">
+      <c r="A17" s="135" t="s">
         <v>96</v>
       </c>
-      <c r="B17" s="131"/>
-      <c r="C17" s="131"/>
-      <c r="D17" s="131"/>
-      <c r="E17" s="132"/>
+      <c r="B17" s="136"/>
+      <c r="C17" s="136"/>
+      <c r="D17" s="136"/>
+      <c r="E17" s="137"/>
       <c r="F17" s="76">
         <f>SUM(F10:F16)</f>
         <v>200</v>
@@ -12303,16 +12303,6 @@
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="G10:O10"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:E12"/>
     <mergeCell ref="B13:C13"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="A17:E17"/>
@@ -12322,6 +12312,16 @@
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="D16:E16"/>
+    <mergeCell ref="A8:F8"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G10:O10"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7 D18" xr:uid="{517DF1E8-3052-48CF-9AE1-C19E6ECB6686}">
@@ -13336,6 +13336,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AD10A028B4ACBB47B37340D8D4079B36" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="436e80374471046821afb96e56969fce">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="606bf0c3-7c02-4ad1-9a2b-bad21eeec9a2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="819cb4b524acab89028d2f2d821df341" ns2:_="">
     <xsd:import namespace="606bf0c3-7c02-4ad1-9a2b-bad21eeec9a2"/>
@@ -13473,22 +13488,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D445429-43EF-4578-A593-6E166DDD94D2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBA7CA51-3876-42E5-9D60-4320955E597F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84037CEB-E5D3-4F40-B93D-B68754BA7EB6}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13506,23 +13523,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BBA7CA51-3876-42E5-9D60-4320955E597F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D445429-43EF-4578-A593-6E166DDD94D2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{5138fff4-6130-46cf-adb5-ec5d984d54d5}" enabled="1" method="Privileged" siteId="{174c7352-9c5c-4558-b848-be140b444e7d}" contentBits="2" removed="0"/>

</xml_diff>